<commit_message>
Publica estado validado de Excel en Ruta
</commit_message>
<xml_diff>
--- a/downloads/exercises/inicial-m07-i07-l03-pr01.xlsx
+++ b/downloads/exercises/inicial-m07-i07-l03-pr01.xlsx
@@ -495,16 +495,12 @@
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="20" t="str">
-        <x:v>Promedio del grupo</x:v>
-      </x:c>
+      <x:c r="A11" s="20" t="str"/>
       <x:c r="B11" s="26" t="str"/>
       <x:c r="C11" s="26" t="str"/>
       <x:c r="D11" s="26" t="str"/>
       <x:c r="E11" s="26" t="str"/>
-      <x:c r="F11" s="20" t="str">
-        <x:v>Calcula también el promedio de los promedios válidos</x:v>
-      </x:c>
+      <x:c r="F11" s="20" t="str"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="20"/>

</xml_diff>